<commit_message>
ordena repo y agrega readme
</commit_message>
<xml_diff>
--- a/output/tablas/tablas informe publicaciones.xlsx
+++ b/output/tablas/tablas informe publicaciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\GitHub\DIP\publicaciones-facso\output\tablas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B769B8DC-9E65-40D6-AB91-85D07ED91E90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B8999B-551A-44CC-AF40-22E5544E8893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{21ABAB56-FFBF-4B2E-9C21-712F2E98FF24}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="10" xr2:uid="{21ABAB56-FFBF-4B2E-9C21-712F2E98FF24}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabla Sintesis" sheetId="9" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="160">
   <si>
     <t>Publicación</t>
   </si>
@@ -75,9 +75,6 @@
     <t>ESTUDIOS ATACAMENOS</t>
   </si>
   <si>
-    <t>MAGALLANIA</t>
-  </si>
-  <si>
     <t>QUATERNARY INTERNATIONAL</t>
   </si>
   <si>
@@ -102,9 +99,6 @@
     <t>Dialogo andino</t>
   </si>
   <si>
-    <t>REVISTA COMPLUTENSE DE EDUCACION</t>
-  </si>
-  <si>
     <t>Psicología</t>
   </si>
   <si>
@@ -141,9 +135,6 @@
     <t>FRONTIERS IN SOCIOLOGY</t>
   </si>
   <si>
-    <t>Revista Chilena de Derecho y Ciencia Política</t>
-  </si>
-  <si>
     <t>Trabajo social</t>
   </si>
   <si>
@@ -171,27 +162,12 @@
     <t>Femenino</t>
   </si>
   <si>
-    <t>3.77</t>
-  </si>
-  <si>
-    <t>3.16</t>
-  </si>
-  <si>
-    <t>0.95</t>
-  </si>
-  <si>
     <t>0.99</t>
   </si>
   <si>
     <t>Masculino</t>
   </si>
   <si>
-    <t>2.58</t>
-  </si>
-  <si>
-    <t>2.29</t>
-  </si>
-  <si>
     <t>0.51</t>
   </si>
   <si>
@@ -204,36 +180,18 @@
     <t>Menos de 50 años</t>
   </si>
   <si>
-    <t>3.47</t>
-  </si>
-  <si>
-    <t>2.72</t>
-  </si>
-  <si>
     <t>0.78</t>
   </si>
   <si>
-    <t>0.59</t>
-  </si>
-  <si>
     <t>50 a 59 años</t>
   </si>
   <si>
-    <t>3.51</t>
-  </si>
-  <si>
-    <t>0.81</t>
-  </si>
-  <si>
     <t>1.07</t>
   </si>
   <si>
     <t>60 años o más</t>
   </si>
   <si>
-    <t>1.76</t>
-  </si>
-  <si>
     <t>1.42</t>
   </si>
   <si>
@@ -249,42 +207,15 @@
     <t>Asistente</t>
   </si>
   <si>
-    <t>1.81</t>
-  </si>
-  <si>
-    <t>1.23</t>
-  </si>
-  <si>
-    <t>0.42</t>
-  </si>
-  <si>
-    <t>0.22</t>
-  </si>
-  <si>
     <t>Asociado</t>
   </si>
   <si>
-    <t>4.12</t>
-  </si>
-  <si>
-    <t>3.82</t>
-  </si>
-  <si>
-    <t>0.98</t>
-  </si>
-  <si>
     <t>Titular</t>
   </si>
   <si>
-    <t>4.18</t>
-  </si>
-  <si>
     <t>3.53</t>
   </si>
   <si>
-    <t>0.84</t>
-  </si>
-  <si>
     <t>1.12</t>
   </si>
   <si>
@@ -324,66 +255,39 @@
     <t>EARLY YEARS</t>
   </si>
   <si>
-    <t>EDUCATION POLICY ANALYSIS ARCHIVES</t>
-  </si>
-  <si>
     <t>BMC PSYCHIATRY</t>
   </si>
   <si>
     <t>INTERNATIONAL JOURNAL OF ENVIRONMENTAL RESEARCH AND PUBLIC HEALTH</t>
   </si>
   <si>
-    <t>JOURNAL OF COMMUNITY PSYCHOLOGY</t>
-  </si>
-  <si>
     <t>LATIN AMERICAN RESEARCH REVIEW</t>
   </si>
   <si>
-    <t>CINTA DE MOEBIO</t>
-  </si>
-  <si>
     <t>CUHSO-CULTURA-HOMBRE-SOCIEDAD</t>
   </si>
   <si>
-    <t>HISTORIA-SANTIAGO</t>
-  </si>
-  <si>
     <t>BRITISH JOURNAL OF SOCIAL WORK</t>
   </si>
   <si>
     <t>AFFILIA-FEMINIST INQUIRY IN SOCIAL WORK</t>
   </si>
   <si>
-    <t>EARTHS FUTURE</t>
-  </si>
-  <si>
     <t>Publicaciones por JCE</t>
   </si>
   <si>
     <t>% Q1+Q2</t>
   </si>
   <si>
-    <t>4.9</t>
-  </si>
-  <si>
     <t>3.1</t>
   </si>
   <si>
-    <t>4.1</t>
-  </si>
-  <si>
     <t>5.0</t>
   </si>
   <si>
     <t>2.1</t>
   </si>
   <si>
-    <t>5.2</t>
-  </si>
-  <si>
-    <t>5.7</t>
-  </si>
-  <si>
     <t>N publicaciones OA</t>
   </si>
   <si>
@@ -408,9 +312,6 @@
     <t>Artículos / capítulos / libros</t>
   </si>
   <si>
-    <t>946 / 171 / 45</t>
-  </si>
-  <si>
     <t>Proporción de artículos</t>
   </si>
   <si>
@@ -423,9 +324,6 @@
     <t>Total de citas / promedio por artículo</t>
   </si>
   <si>
-    <t>4.854 / 6,7</t>
-  </si>
-  <si>
     <t>Índice h institucional</t>
   </si>
   <si>
@@ -508,6 +406,129 @@
   </si>
   <si>
     <t>Idioma</t>
+  </si>
+  <si>
+    <t>900 / 161 / 43</t>
+  </si>
+  <si>
+    <t>4.773 / 7,47</t>
+  </si>
+  <si>
+    <t>LATIN AMERICAN ANTIQUITY</t>
+  </si>
+  <si>
+    <t>INTERCIENCIA</t>
+  </si>
+  <si>
+    <t>REVISTA AUSTRAL DE CIENCIAS SOCIALES</t>
+  </si>
+  <si>
+    <t>2.91</t>
+  </si>
+  <si>
+    <t>0.90</t>
+  </si>
+  <si>
+    <t>1.01</t>
+  </si>
+  <si>
+    <t>2.62</t>
+  </si>
+  <si>
+    <t>2.20</t>
+  </si>
+  <si>
+    <t>3.45</t>
+  </si>
+  <si>
+    <t>2.57</t>
+  </si>
+  <si>
+    <t>3.54</t>
+  </si>
+  <si>
+    <t>3.22</t>
+  </si>
+  <si>
+    <t>0.74</t>
+  </si>
+  <si>
+    <t>1.78</t>
+  </si>
+  <si>
+    <t>1.68</t>
+  </si>
+  <si>
+    <t>1.16</t>
+  </si>
+  <si>
+    <t>0.40</t>
+  </si>
+  <si>
+    <t>0.24</t>
+  </si>
+  <si>
+    <t>4.04</t>
+  </si>
+  <si>
+    <t>3.58</t>
+  </si>
+  <si>
+    <t>0.94</t>
+  </si>
+  <si>
+    <t>4.09</t>
+  </si>
+  <si>
+    <t>3.33</t>
+  </si>
+  <si>
+    <t>0.80</t>
+  </si>
+  <si>
+    <t>Porcentaje</t>
+  </si>
+  <si>
+    <t>Q3</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>INTERNATIONAL JOURNAL OF EARLY CHILDHOOD</t>
+  </si>
+  <si>
+    <t>RLA-REVISTA DE LINGUISTICA TEORICA Y APLICADA</t>
+  </si>
+  <si>
+    <t>ESTUDIOS FILOLOGICOS</t>
+  </si>
+  <si>
+    <t>LEARNING AND MOTIVATION</t>
+  </si>
+  <si>
+    <t>CURRENT SOCIOLOGY</t>
+  </si>
+  <si>
+    <t>International Labour Review</t>
+  </si>
+  <si>
+    <t>REVISTA DE ESTUDIOS SOCIALES</t>
+  </si>
+  <si>
+    <t>4.6</t>
+  </si>
+  <si>
+    <t>4.0</t>
+  </si>
+  <si>
+    <t>4.7</t>
+  </si>
+  <si>
+    <t>1.9</t>
+  </si>
+  <si>
+    <t>5.6</t>
   </si>
 </sst>
 </file>
@@ -537,14 +558,14 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="13"/>
+      <color rgb="FF151618"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <sz val="13"/>
+      <color rgb="FF151618"/>
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
@@ -621,7 +642,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -671,35 +692,41 @@
     <xf numFmtId="9" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1044,100 +1071,100 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="17.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="23" t="s">
-        <v>114</v>
+        <v>82</v>
       </c>
       <c r="B2" s="24" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="19" t="s">
-        <v>116</v>
+        <v>84</v>
       </c>
       <c r="B3" s="20">
-        <v>1162</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="19" t="s">
-        <v>117</v>
+        <v>85</v>
       </c>
       <c r="B4" s="20">
-        <v>1328</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>1273</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
-        <v>118</v>
+        <v>86</v>
       </c>
       <c r="B5" s="21" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="19" t="s">
-        <v>120</v>
+        <v>87</v>
       </c>
       <c r="B6" s="22">
         <v>0.81</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="19" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="B7" s="21">
-        <v>7.8</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>7.41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="19" t="s">
-        <v>121</v>
+        <v>88</v>
       </c>
       <c r="B8" s="22">
         <v>0.78</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="19" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="B9" s="22">
-        <v>0.67</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="83.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="19" t="s">
-        <v>123</v>
+        <v>90</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="50.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="19" t="s">
-        <v>125</v>
+        <v>91</v>
       </c>
       <c r="B11" s="21">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="99.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="38.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="19" t="s">
-        <v>126</v>
+        <v>92</v>
       </c>
       <c r="B12" s="22">
-        <v>0.49</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="66.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="25" t="s">
-        <v>127</v>
+        <v>93</v>
       </c>
       <c r="B13" s="26">
         <v>0.45</v>
@@ -1145,6 +1172,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1158,28 +1186,28 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>102</v>
+        <v>74</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>103</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
+      <c r="A2" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
     </row>
     <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="7" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>104</v>
+        <v>155</v>
       </c>
       <c r="C3" s="10">
         <v>0.71</v>
@@ -1187,93 +1215,93 @@
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="7" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>105</v>
+        <v>76</v>
       </c>
       <c r="C4" s="10">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
+      <c r="A5" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
     </row>
     <row r="6" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>106</v>
+        <v>156</v>
       </c>
       <c r="C6" s="10">
-        <v>0.66</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>107</v>
+        <v>157</v>
       </c>
       <c r="C7" s="10">
-        <v>0.68</v>
+        <v>0.69</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="7" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="C8" s="10">
         <v>0.65</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
+      <c r="A9" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
     </row>
     <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="7" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>108</v>
+        <v>158</v>
       </c>
       <c r="C10" s="10">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="7" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>109</v>
+        <v>77</v>
       </c>
       <c r="C11" s="10">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>110</v>
+        <v>159</v>
       </c>
       <c r="C12" s="12">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
     </row>
   </sheetData>
@@ -1297,138 +1325,138 @@
   <sheetData>
     <row r="1" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>112</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
-        <v>79</v>
-      </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
+      <c r="A2" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="18"/>
     </row>
     <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C3" s="13">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4" s="2">
         <v>18</v>
       </c>
       <c r="C4" s="13">
-        <v>0.47</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C5" s="13">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B6" s="2">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="C6" s="13">
-        <v>0.52</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B7" s="2">
-        <v>81</v>
+        <v>71</v>
       </c>
       <c r="C7" s="13">
-        <v>0.56000000000000005</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="17"/>
-      <c r="C8" s="17"/>
+      <c r="A8" s="18" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="18"/>
+      <c r="C8" s="18"/>
     </row>
     <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B9" s="2">
-        <v>242</v>
+        <v>220</v>
       </c>
       <c r="C9" s="13">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B10" s="2">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C10" s="13">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
+      <c r="A11" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="18"/>
     </row>
     <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B12" s="2">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="C12" s="13">
-        <v>0.41</v>
+        <v>0.4</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B13" s="2">
-        <v>241</v>
+        <v>218</v>
       </c>
       <c r="C13" s="13">
-        <v>0.53</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B14" s="2">
         <v>57</v>
@@ -1438,40 +1466,40 @@
       </c>
     </row>
     <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="B15" s="17"/>
-      <c r="C15" s="17"/>
+      <c r="A15" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" s="18"/>
+      <c r="C15" s="18"/>
     </row>
     <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B16" s="2">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="C16" s="13">
-        <v>0.4</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="B17" s="2">
-        <v>270</v>
+        <v>250</v>
       </c>
       <c r="C17" s="13">
-        <v>0.53</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="B18" s="6">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C18" s="16">
         <v>0.43</v>
@@ -1498,168 +1526,168 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>128</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>129</v>
-      </c>
-      <c r="B2" s="18"/>
+      <c r="A2" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="B2" s="17"/>
     </row>
     <row r="3" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>129</v>
+        <v>95</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>130</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="18" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="18"/>
-    </row>
-    <row r="5" spans="1:2" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="17"/>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>131</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>132</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>133</v>
+        <v>99</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>134</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>135</v>
+        <v>101</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>136</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>137</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="B11" s="18"/>
+      <c r="A11" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="17"/>
     </row>
     <row r="12" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>138</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B14" s="17"/>
+    </row>
+    <row r="15" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B13" s="7" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="B14" s="18"/>
-    </row>
-    <row r="15" spans="1:2" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
+      <c r="B16" s="7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="B15" s="7" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="B18" s="18"/>
+      <c r="B18" s="17"/>
     </row>
     <row r="19" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>143</v>
+        <v>109</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>144</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>145</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>146</v>
+        <v>112</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>147</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1684,10 +1712,10 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>148</v>
+        <v>114</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>149</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1695,39 +1723,39 @@
         <v>1</v>
       </c>
       <c r="B2" s="7">
-        <v>937</v>
+        <v>895</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="B3" s="7">
-        <v>736</v>
+        <v>694</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="B4" s="7">
-        <v>703</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>151</v>
+        <v>117</v>
       </c>
       <c r="B5" s="7">
-        <v>737</v>
+        <v>692</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>152</v>
+        <v>118</v>
       </c>
       <c r="B6" s="9">
-        <v>829</v>
+        <v>781</v>
       </c>
     </row>
   </sheetData>
@@ -1755,13 +1783,13 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-    </row>
-    <row r="3" spans="1:3" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1769,10 +1797,10 @@
         <v>5</v>
       </c>
       <c r="C3" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="86.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1783,20 +1811,20 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>7</v>
+        <v>121</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>5</v>
@@ -1805,9 +1833,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>5</v>
@@ -1817,40 +1845,40 @@
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-    </row>
-    <row r="9" spans="1:3" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>11</v>
+        <v>122</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
+      <c r="B10" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C11" s="2">
         <v>4</v>
@@ -1858,50 +1886,50 @@
     </row>
     <row r="12" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C12" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
+      <c r="A14" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
     </row>
     <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C16" s="2">
         <v>8</v>
@@ -1909,10 +1937,10 @@
     </row>
     <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C17" s="2">
         <v>6</v>
@@ -1920,18 +1948,18 @@
     </row>
     <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="C18" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>5</v>
@@ -1941,18 +1969,18 @@
       </c>
     </row>
     <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
+      <c r="A20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
     </row>
     <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C21" s="2">
         <v>7</v>
@@ -1960,10 +1988,10 @@
     </row>
     <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="C22" s="2">
         <v>7</v>
@@ -1971,50 +1999,50 @@
     </row>
     <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C23" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>29</v>
+        <v>123</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C24" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C25" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
+      <c r="A26" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
     </row>
     <row r="27" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C27" s="2">
         <v>24</v>
@@ -2022,10 +2050,10 @@
     </row>
     <row r="28" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C28" s="2">
         <v>10</v>
@@ -2033,10 +2061,10 @@
     </row>
     <row r="29" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" s="2">
         <v>6</v>
@@ -2044,21 +2072,21 @@
     </row>
     <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C30" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C31" s="6">
         <v>4</v>
@@ -2083,182 +2111,182 @@
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>5</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>38</v>
-      </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+      <c r="A2" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
     </row>
     <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>41</v>
+        <v>124</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>42</v>
+        <v>125</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>43</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>45</v>
+        <v>127</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>46</v>
+        <v>128</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
+      <c r="A5" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
     </row>
     <row r="6" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>51</v>
+        <v>129</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>52</v>
+        <v>130</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>54</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>40</v>
+        <v>131</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>56</v>
+        <v>132</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>57</v>
+        <v>133</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>58</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>60</v>
+        <v>134</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>62</v>
+        <v>48</v>
       </c>
       <c r="E8" s="7" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
-        <v>64</v>
-      </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
-      <c r="E9" s="18"/>
+      <c r="A9" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
     </row>
     <row r="10" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>66</v>
+        <v>135</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>67</v>
+        <v>136</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>68</v>
+        <v>137</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>69</v>
+        <v>138</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>71</v>
+        <v>139</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>72</v>
+        <v>140</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>73</v>
+        <v>141</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>75</v>
+        <v>142</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>76</v>
+        <v>143</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>77</v>
+        <v>144</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -2281,16 +2309,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2298,10 +2326,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="7">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C2" s="7">
-        <v>1169</v>
+        <v>1186</v>
       </c>
       <c r="D2" s="7">
         <v>16</v>
@@ -2309,13 +2337,13 @@
     </row>
     <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B3" s="7">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C3" s="7">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D3" s="7">
         <v>5</v>
@@ -2323,13 +2351,13 @@
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B4" s="7">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="C4" s="7">
-        <v>2148</v>
+        <v>2165</v>
       </c>
       <c r="D4" s="7">
         <v>22</v>
@@ -2337,10 +2365,10 @@
     </row>
     <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B5" s="7">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C5" s="7">
         <v>951</v>
@@ -2349,18 +2377,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B6" s="9">
-        <v>139</v>
+        <v>121</v>
       </c>
       <c r="C6" s="9">
-        <v>774</v>
+        <v>662</v>
       </c>
       <c r="D6" s="9">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -2375,35 +2403,35 @@
   <sheetData>
     <row r="1" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>81</v>
+        <v>58</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>82</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
+      <c r="A2" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
     </row>
     <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B3" s="7">
-        <v>464</v>
+        <v>431</v>
       </c>
       <c r="C3" s="7">
-        <v>3566</v>
+        <v>3444</v>
       </c>
       <c r="D3" s="7">
         <v>26</v>
@@ -2411,35 +2439,35 @@
     </row>
     <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B4" s="7">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="C4" s="7">
-        <v>2121</v>
+        <v>2167</v>
       </c>
       <c r="D4" s="7">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
+    <row r="5" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="17"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
     </row>
     <row r="6" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B6" s="7">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="C6" s="7">
-        <v>1361</v>
+        <v>1386</v>
       </c>
       <c r="D6" s="7">
         <v>16</v>
@@ -2447,49 +2475,49 @@
     </row>
     <row r="7" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="B7" s="7">
-        <v>426</v>
+        <v>396</v>
       </c>
       <c r="C7" s="7">
-        <v>3449</v>
+        <v>3336</v>
       </c>
       <c r="D7" s="7">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="B8" s="7">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C8" s="7">
-        <v>877</v>
+        <v>889</v>
       </c>
       <c r="D8" s="7">
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="B9" s="18"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="18"/>
+    <row r="9" spans="1:4" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
     </row>
     <row r="10" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="B10" s="7">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="C10" s="7">
-        <v>792</v>
+        <v>714</v>
       </c>
       <c r="D10" s="7">
         <v>12</v>
@@ -2497,27 +2525,27 @@
     </row>
     <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>70</v>
+        <v>52</v>
       </c>
       <c r="B11" s="7">
-        <v>473</v>
+        <v>456</v>
       </c>
       <c r="C11" s="7">
-        <v>3553</v>
+        <v>3556</v>
       </c>
       <c r="D11" s="7">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
       <c r="B12" s="9">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="C12" s="9">
-        <v>1341</v>
+        <v>1339</v>
       </c>
       <c r="D12" s="9">
         <v>17</v>
@@ -2535,9 +2563,65 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70DFFA49-4802-44AA-8A4B-8521AA5C61B8}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="2">
+        <v>306</v>
+      </c>
+      <c r="C2" s="27">
+        <v>0.439</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="2">
+        <v>171</v>
+      </c>
+      <c r="C3" s="27">
+        <v>0.245</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" s="2">
+        <v>166</v>
+      </c>
+      <c r="C4" s="27">
+        <v>0.23799999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" s="6">
+        <v>54</v>
+      </c>
+      <c r="C5" s="28">
+        <v>7.6999999999999999E-2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2555,149 +2639,149 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-    </row>
-    <row r="3" spans="1:3" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+    </row>
+    <row r="3" spans="1:3" ht="72" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="C3" s="2">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="86.25" thickBot="1" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="86.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C4" s="2">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="43.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C5" s="2">
         <v>7</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="C5" s="2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:3" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="C6" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="57.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="C7" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="18"/>
-    </row>
-    <row r="9" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
+    </row>
+    <row r="9" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C9" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="C10" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>35</v>
+        <v>148</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="C11" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>91</v>
+        <v>149</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="C12" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>21</v>
+        <v>150</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="C13" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="18" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="18"/>
+      <c r="A14" s="17" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="17"/>
+      <c r="C14" s="17"/>
     </row>
     <row r="15" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="C15" s="2">
         <v>6</v>
@@ -2705,61 +2789,61 @@
     </row>
     <row r="16" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>68</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C16" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C17" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>93</v>
+        <v>21</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C18" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>94</v>
+        <v>151</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C19" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="18"/>
-      <c r="C20" s="18"/>
+      <c r="A20" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
     </row>
     <row r="21" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C21" s="2">
         <v>4</v>
@@ -2767,10 +2851,10 @@
     </row>
     <row r="22" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C22" s="2">
         <v>3</v>
@@ -2778,10 +2862,10 @@
     </row>
     <row r="23" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="C23" s="2">
         <v>3</v>
@@ -2789,50 +2873,50 @@
     </row>
     <row r="24" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>97</v>
+        <v>152</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>88</v>
+        <v>66</v>
       </c>
       <c r="C24" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>98</v>
+        <v>153</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>89</v>
+        <v>65</v>
       </c>
       <c r="C25" s="2">
         <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
+      <c r="A26" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
     </row>
     <row r="27" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C27" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C28" s="2">
         <v>4</v>
@@ -2840,32 +2924,32 @@
     </row>
     <row r="29" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
-        <v>99</v>
+        <v>154</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C29" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C30" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>101</v>
+        <v>32</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C31" s="6">
         <v>3</v>

</xml_diff>